<commit_message>
fix rozen excel start row
</commit_message>
<xml_diff>
--- a/public/templates/rozen_template.xlsx
+++ b/public/templates/rozen_template.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ruru/Desktop/일일정산표/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0F695FC-36C7-DB40-A727-899C5575A88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="75" windowWidth="21360" windowHeight="12495"/>
+    <workbookView xWindow="360" yWindow="680" windowWidth="21360" windowHeight="12500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="엑셀파일 첫행-제목없음" sheetId="1" r:id="rId1"/>
@@ -17,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="26">
   <si>
     <t>수하인명</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -125,8 +131,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <name val="돋움"/>
@@ -198,14 +204,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -243,7 +252,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -315,7 +324,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -488,81 +497,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="H1:H2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="5.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="32.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="3.21875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.88671875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="4.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="3.1640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.83203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="4.1640625" style="1" customWidth="1"/>
     <col min="9" max="9" width="16.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="5.109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.21875" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="10" max="10" width="5.1640625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.1640625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="1">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2500</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="1">
-        <v>2</v>
-      </c>
-      <c r="G2" s="1">
-        <v>6000</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>5</v>
-      </c>
+    <row r="1" spans="8:8">
+      <c r="H1" s="2"/>
+    </row>
+    <row r="2" spans="8:8">
+      <c r="H2" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -573,25 +530,25 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="5.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="31.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="6.21875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="7.109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="6.5546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.44140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="3.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="1"/>
+    <col min="2" max="2" width="5.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="6.1640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="7.1640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5" style="1" customWidth="1"/>
+    <col min="10" max="10" width="3.1640625" style="1" customWidth="1"/>
     <col min="11" max="11" width="23" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="12" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:11">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -622,7 +579,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:11">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -651,7 +608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:11">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -688,22 +645,22 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="6.109375" customWidth="1"/>
+    <col min="1" max="1" width="6.1640625" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" customWidth="1"/>
-    <col min="5" max="6" width="9.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" customWidth="1"/>
+    <col min="5" max="6" width="9.5" customWidth="1"/>
     <col min="7" max="7" width="5.33203125" customWidth="1"/>
-    <col min="9" max="9" width="5.109375" customWidth="1"/>
+    <col min="9" max="9" width="5.1640625" customWidth="1"/>
     <col min="10" max="10" width="14.6640625" customWidth="1"/>
-    <col min="12" max="12" width="17.21875" customWidth="1"/>
+    <col min="12" max="12" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -738,7 +695,7 @@
       </c>
       <c r="M1" s="1"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -781,21 +738,21 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="2" max="2" width="6.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" customWidth="1"/>
-    <col min="6" max="6" width="12.21875" customWidth="1"/>
-    <col min="10" max="10" width="17.109375" customWidth="1"/>
-    <col min="11" max="11" width="3.5546875" customWidth="1"/>
-    <col min="12" max="12" width="17.88671875" customWidth="1"/>
+    <col min="2" max="2" width="6.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" customWidth="1"/>
+    <col min="4" max="4" width="15.5" customWidth="1"/>
+    <col min="5" max="5" width="11.5" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" customWidth="1"/>
+    <col min="10" max="10" width="17.1640625" customWidth="1"/>
+    <col min="11" max="11" width="3.5" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -829,7 +786,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -863,7 +820,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>

</xml_diff>